<commit_message>
Fix master table: drop 386 blank padding rows inherited from Level4
</commit_message>
<xml_diff>
--- a/terrestrial/Towards_SDS/Terrestrial_Master_SDS-aligned.xlsx
+++ b/terrestrial/Towards_SDS/Terrestrial_Master_SDS-aligned.xlsx
@@ -10,7 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="tblGeoschemesTerrestrial" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'tblGeoschemesTerrestrial'!$A$1:$M$1435</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'tblGeoschemesTerrestrial'!$A$1:$M$1049</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -428,7 +428,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M1435"/>
+  <dimension ref="A1:M1049"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -31954,1938 +31954,8 @@
         </is>
       </c>
     </row>
-    <row r="1050">
-      <c r="A1050" t="n">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="1051">
-      <c r="A1051" t="n">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="1052">
-      <c r="A1052" t="n">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="1053">
-      <c r="A1053" t="n">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="1054">
-      <c r="A1054" t="n">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="1055">
-      <c r="A1055" t="n">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="1056">
-      <c r="A1056" t="n">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="1057">
-      <c r="A1057" t="n">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="1058">
-      <c r="A1058" t="n">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="1059">
-      <c r="A1059" t="n">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="1060">
-      <c r="A1060" t="n">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="1061">
-      <c r="A1061" t="n">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="1062">
-      <c r="A1062" t="n">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="1063">
-      <c r="A1063" t="n">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="1064">
-      <c r="A1064" t="n">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="1065">
-      <c r="A1065" t="n">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="1066">
-      <c r="A1066" t="n">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="1067">
-      <c r="A1067" t="n">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="1068">
-      <c r="A1068" t="n">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="1069">
-      <c r="A1069" t="n">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="1070">
-      <c r="A1070" t="n">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="1071">
-      <c r="A1071" t="n">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="1072">
-      <c r="A1072" t="n">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="1073">
-      <c r="A1073" t="n">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="1074">
-      <c r="A1074" t="n">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="1075">
-      <c r="A1075" t="n">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="1076">
-      <c r="A1076" t="n">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="1077">
-      <c r="A1077" t="n">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="1078">
-      <c r="A1078" t="n">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="1079">
-      <c r="A1079" t="n">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="1080">
-      <c r="A1080" t="n">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="1081">
-      <c r="A1081" t="n">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="1082">
-      <c r="A1082" t="n">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="1083">
-      <c r="A1083" t="n">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="1084">
-      <c r="A1084" t="n">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="1085">
-      <c r="A1085" t="n">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="1086">
-      <c r="A1086" t="n">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="1087">
-      <c r="A1087" t="n">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="1088">
-      <c r="A1088" t="n">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="1089">
-      <c r="A1089" t="n">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="1090">
-      <c r="A1090" t="n">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="1091">
-      <c r="A1091" t="n">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="1092">
-      <c r="A1092" t="n">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="1093">
-      <c r="A1093" t="n">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="1094">
-      <c r="A1094" t="n">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="1095">
-      <c r="A1095" t="n">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="1096">
-      <c r="A1096" t="n">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="1097">
-      <c r="A1097" t="n">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="1098">
-      <c r="A1098" t="n">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="1099">
-      <c r="A1099" t="n">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="1100">
-      <c r="A1100" t="n">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="1101">
-      <c r="A1101" t="n">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="1102">
-      <c r="A1102" t="n">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="1103">
-      <c r="A1103" t="n">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="1104">
-      <c r="A1104" t="n">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="1105">
-      <c r="A1105" t="n">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="1106">
-      <c r="A1106" t="n">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="1107">
-      <c r="A1107" t="n">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="1108">
-      <c r="A1108" t="n">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="1109">
-      <c r="A1109" t="n">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="1110">
-      <c r="A1110" t="n">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="1111">
-      <c r="A1111" t="n">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="1112">
-      <c r="A1112" t="n">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="1113">
-      <c r="A1113" t="n">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="1114">
-      <c r="A1114" t="n">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="1115">
-      <c r="A1115" t="n">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="1116">
-      <c r="A1116" t="n">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="1117">
-      <c r="A1117" t="n">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="1118">
-      <c r="A1118" t="n">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="1119">
-      <c r="A1119" t="n">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="1120">
-      <c r="A1120" t="n">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="1121">
-      <c r="A1121" t="n">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="1122">
-      <c r="A1122" t="n">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="1123">
-      <c r="A1123" t="n">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="1124">
-      <c r="A1124" t="n">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="1125">
-      <c r="A1125" t="n">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="1126">
-      <c r="A1126" t="n">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="1127">
-      <c r="A1127" t="n">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="1128">
-      <c r="A1128" t="n">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="1129">
-      <c r="A1129" t="n">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="1130">
-      <c r="A1130" t="n">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="1131">
-      <c r="A1131" t="n">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="1132">
-      <c r="A1132" t="n">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="1133">
-      <c r="A1133" t="n">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="1134">
-      <c r="A1134" t="n">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="1135">
-      <c r="A1135" t="n">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="1136">
-      <c r="A1136" t="n">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="1137">
-      <c r="A1137" t="n">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="1138">
-      <c r="A1138" t="n">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="1139">
-      <c r="A1139" t="n">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="1140">
-      <c r="A1140" t="n">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="1141">
-      <c r="A1141" t="n">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="1142">
-      <c r="A1142" t="n">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="1143">
-      <c r="A1143" t="n">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="1144">
-      <c r="A1144" t="n">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="1145">
-      <c r="A1145" t="n">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="1146">
-      <c r="A1146" t="n">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="1147">
-      <c r="A1147" t="n">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="1148">
-      <c r="A1148" t="n">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="1149">
-      <c r="A1149" t="n">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="1150">
-      <c r="A1150" t="n">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="1151">
-      <c r="A1151" t="n">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="1152">
-      <c r="A1152" t="n">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="1153">
-      <c r="A1153" t="n">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="1154">
-      <c r="A1154" t="n">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="1155">
-      <c r="A1155" t="n">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="1156">
-      <c r="A1156" t="n">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="1157">
-      <c r="A1157" t="n">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="1158">
-      <c r="A1158" t="n">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="1159">
-      <c r="A1159" t="n">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="1160">
-      <c r="A1160" t="n">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="1161">
-      <c r="A1161" t="n">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="1162">
-      <c r="A1162" t="n">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="1163">
-      <c r="A1163" t="n">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="1164">
-      <c r="A1164" t="n">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="1165">
-      <c r="A1165" t="n">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="1166">
-      <c r="A1166" t="n">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="1167">
-      <c r="A1167" t="n">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="1168">
-      <c r="A1168" t="n">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="1169">
-      <c r="A1169" t="n">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="1170">
-      <c r="A1170" t="n">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="1171">
-      <c r="A1171" t="n">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="1172">
-      <c r="A1172" t="n">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="1173">
-      <c r="A1173" t="n">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="1174">
-      <c r="A1174" t="n">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="1175">
-      <c r="A1175" t="n">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="1176">
-      <c r="A1176" t="n">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="1177">
-      <c r="A1177" t="n">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="1178">
-      <c r="A1178" t="n">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="1179">
-      <c r="A1179" t="n">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="1180">
-      <c r="A1180" t="n">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="1181">
-      <c r="A1181" t="n">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="1182">
-      <c r="A1182" t="n">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="1183">
-      <c r="A1183" t="n">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="1184">
-      <c r="A1184" t="n">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="1185">
-      <c r="A1185" t="n">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="1186">
-      <c r="A1186" t="n">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="1187">
-      <c r="A1187" t="n">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="1188">
-      <c r="A1188" t="n">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="1189">
-      <c r="A1189" t="n">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="1190">
-      <c r="A1190" t="n">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="1191">
-      <c r="A1191" t="n">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="1192">
-      <c r="A1192" t="n">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="1193">
-      <c r="A1193" t="n">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="1194">
-      <c r="A1194" t="n">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="1195">
-      <c r="A1195" t="n">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="1196">
-      <c r="A1196" t="n">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="1197">
-      <c r="A1197" t="n">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="1198">
-      <c r="A1198" t="n">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="1199">
-      <c r="A1199" t="n">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="1200">
-      <c r="A1200" t="n">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="1201">
-      <c r="A1201" t="n">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="1202">
-      <c r="A1202" t="n">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="1203">
-      <c r="A1203" t="n">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="1204">
-      <c r="A1204" t="n">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="1205">
-      <c r="A1205" t="n">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="1206">
-      <c r="A1206" t="n">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="1207">
-      <c r="A1207" t="n">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="1208">
-      <c r="A1208" t="n">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="1209">
-      <c r="A1209" t="n">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="1210">
-      <c r="A1210" t="n">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="1211">
-      <c r="A1211" t="n">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="1212">
-      <c r="A1212" t="n">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="1213">
-      <c r="A1213" t="n">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="1214">
-      <c r="A1214" t="n">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="1215">
-      <c r="A1215" t="n">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="1216">
-      <c r="A1216" t="n">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="1217">
-      <c r="A1217" t="n">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="1218">
-      <c r="A1218" t="n">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="1219">
-      <c r="A1219" t="n">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="1220">
-      <c r="A1220" t="n">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="1221">
-      <c r="A1221" t="n">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="1222">
-      <c r="A1222" t="n">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="1223">
-      <c r="A1223" t="n">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="1224">
-      <c r="A1224" t="n">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="1225">
-      <c r="A1225" t="n">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="1226">
-      <c r="A1226" t="n">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="1227">
-      <c r="A1227" t="n">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="1228">
-      <c r="A1228" t="n">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="1229">
-      <c r="A1229" t="n">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="1230">
-      <c r="A1230" t="n">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="1231">
-      <c r="A1231" t="n">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="1232">
-      <c r="A1232" t="n">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="1233">
-      <c r="A1233" t="n">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="1234">
-      <c r="A1234" t="n">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="1235">
-      <c r="A1235" t="n">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="1236">
-      <c r="A1236" t="n">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="1237">
-      <c r="A1237" t="n">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="1238">
-      <c r="A1238" t="n">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="1239">
-      <c r="A1239" t="n">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="1240">
-      <c r="A1240" t="n">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="1241">
-      <c r="A1241" t="n">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="1242">
-      <c r="A1242" t="n">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="1243">
-      <c r="A1243" t="n">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="1244">
-      <c r="A1244" t="n">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="1245">
-      <c r="A1245" t="n">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="1246">
-      <c r="A1246" t="n">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="1247">
-      <c r="A1247" t="n">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="1248">
-      <c r="A1248" t="n">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="1249">
-      <c r="A1249" t="n">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="1250">
-      <c r="A1250" t="n">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="1251">
-      <c r="A1251" t="n">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="1252">
-      <c r="A1252" t="n">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="1253">
-      <c r="A1253" t="n">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="1254">
-      <c r="A1254" t="n">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="1255">
-      <c r="A1255" t="n">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="1256">
-      <c r="A1256" t="n">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="1257">
-      <c r="A1257" t="n">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="1258">
-      <c r="A1258" t="n">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="1259">
-      <c r="A1259" t="n">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="1260">
-      <c r="A1260" t="n">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="1261">
-      <c r="A1261" t="n">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="1262">
-      <c r="A1262" t="n">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="1263">
-      <c r="A1263" t="n">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="1264">
-      <c r="A1264" t="n">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="1265">
-      <c r="A1265" t="n">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="1266">
-      <c r="A1266" t="n">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="1267">
-      <c r="A1267" t="n">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="1268">
-      <c r="A1268" t="n">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="1269">
-      <c r="A1269" t="n">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="1270">
-      <c r="A1270" t="n">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="1271">
-      <c r="A1271" t="n">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="1272">
-      <c r="A1272" t="n">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="1273">
-      <c r="A1273" t="n">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="1274">
-      <c r="A1274" t="n">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="1275">
-      <c r="A1275" t="n">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="1276">
-      <c r="A1276" t="n">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="1277">
-      <c r="A1277" t="n">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="1278">
-      <c r="A1278" t="n">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="1279">
-      <c r="A1279" t="n">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="1280">
-      <c r="A1280" t="n">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="1281">
-      <c r="A1281" t="n">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="1282">
-      <c r="A1282" t="n">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="1283">
-      <c r="A1283" t="n">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="1284">
-      <c r="A1284" t="n">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="1285">
-      <c r="A1285" t="n">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="1286">
-      <c r="A1286" t="n">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="1287">
-      <c r="A1287" t="n">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="1288">
-      <c r="A1288" t="n">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="1289">
-      <c r="A1289" t="n">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="1290">
-      <c r="A1290" t="n">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="1291">
-      <c r="A1291" t="n">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="1292">
-      <c r="A1292" t="n">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="1293">
-      <c r="A1293" t="n">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="1294">
-      <c r="A1294" t="n">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="1295">
-      <c r="A1295" t="n">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="1296">
-      <c r="A1296" t="n">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="1297">
-      <c r="A1297" t="n">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="1298">
-      <c r="A1298" t="n">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="1299">
-      <c r="A1299" t="n">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="1300">
-      <c r="A1300" t="n">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="1301">
-      <c r="A1301" t="n">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="1302">
-      <c r="A1302" t="n">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="1303">
-      <c r="A1303" t="n">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="1304">
-      <c r="A1304" t="n">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="1305">
-      <c r="A1305" t="n">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="1306">
-      <c r="A1306" t="n">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="1307">
-      <c r="A1307" t="n">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="1308">
-      <c r="A1308" t="n">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="1309">
-      <c r="A1309" t="n">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="1310">
-      <c r="A1310" t="n">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="1311">
-      <c r="A1311" t="n">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="1312">
-      <c r="A1312" t="n">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="1313">
-      <c r="A1313" t="n">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="1314">
-      <c r="A1314" t="n">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="1315">
-      <c r="A1315" t="n">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="1316">
-      <c r="A1316" t="n">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="1317">
-      <c r="A1317" t="n">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="1318">
-      <c r="A1318" t="n">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="1319">
-      <c r="A1319" t="n">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="1320">
-      <c r="A1320" t="n">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="1321">
-      <c r="A1321" t="n">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="1322">
-      <c r="A1322" t="n">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="1323">
-      <c r="A1323" t="n">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="1324">
-      <c r="A1324" t="n">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="1325">
-      <c r="A1325" t="n">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="1326">
-      <c r="A1326" t="n">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="1327">
-      <c r="A1327" t="n">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="1328">
-      <c r="A1328" t="n">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="1329">
-      <c r="A1329" t="n">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="1330">
-      <c r="A1330" t="n">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="1331">
-      <c r="A1331" t="n">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="1332">
-      <c r="A1332" t="n">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="1333">
-      <c r="A1333" t="n">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="1334">
-      <c r="A1334" t="n">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="1335">
-      <c r="A1335" t="n">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="1336">
-      <c r="A1336" t="n">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="1337">
-      <c r="A1337" t="n">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="1338">
-      <c r="A1338" t="n">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="1339">
-      <c r="A1339" t="n">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="1340">
-      <c r="A1340" t="n">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="1341">
-      <c r="A1341" t="n">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="1342">
-      <c r="A1342" t="n">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="1343">
-      <c r="A1343" t="n">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="1344">
-      <c r="A1344" t="n">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="1345">
-      <c r="A1345" t="n">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="1346">
-      <c r="A1346" t="n">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="1347">
-      <c r="A1347" t="n">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="1348">
-      <c r="A1348" t="n">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="1349">
-      <c r="A1349" t="n">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="1350">
-      <c r="A1350" t="n">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="1351">
-      <c r="A1351" t="n">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="1352">
-      <c r="A1352" t="n">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="1353">
-      <c r="A1353" t="n">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="1354">
-      <c r="A1354" t="n">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="1355">
-      <c r="A1355" t="n">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="1356">
-      <c r="A1356" t="n">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="1357">
-      <c r="A1357" t="n">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="1358">
-      <c r="A1358" t="n">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="1359">
-      <c r="A1359" t="n">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="1360">
-      <c r="A1360" t="n">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="1361">
-      <c r="A1361" t="n">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="1362">
-      <c r="A1362" t="n">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="1363">
-      <c r="A1363" t="n">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="1364">
-      <c r="A1364" t="n">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="1365">
-      <c r="A1365" t="n">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="1366">
-      <c r="A1366" t="n">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="1367">
-      <c r="A1367" t="n">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="1368">
-      <c r="A1368" t="n">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="1369">
-      <c r="A1369" t="n">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="1370">
-      <c r="A1370" t="n">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="1371">
-      <c r="A1371" t="n">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="1372">
-      <c r="A1372" t="n">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="1373">
-      <c r="A1373" t="n">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="1374">
-      <c r="A1374" t="n">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="1375">
-      <c r="A1375" t="n">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="1376">
-      <c r="A1376" t="n">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="1377">
-      <c r="A1377" t="n">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="1378">
-      <c r="A1378" t="n">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="1379">
-      <c r="A1379" t="n">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="1380">
-      <c r="A1380" t="n">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="1381">
-      <c r="A1381" t="n">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="1382">
-      <c r="A1382" t="n">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="1383">
-      <c r="A1383" t="n">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="1384">
-      <c r="A1384" t="n">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="1385">
-      <c r="A1385" t="n">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="1386">
-      <c r="A1386" t="n">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="1387">
-      <c r="A1387" t="n">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="1388">
-      <c r="A1388" t="n">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="1389">
-      <c r="A1389" t="n">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="1390">
-      <c r="A1390" t="n">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="1391">
-      <c r="A1391" t="n">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="1392">
-      <c r="A1392" t="n">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="1393">
-      <c r="A1393" t="n">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="1394">
-      <c r="A1394" t="n">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="1395">
-      <c r="A1395" t="n">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="1396">
-      <c r="A1396" t="n">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="1397">
-      <c r="A1397" t="n">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="1398">
-      <c r="A1398" t="n">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="1399">
-      <c r="A1399" t="n">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="1400">
-      <c r="A1400" t="n">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="1401">
-      <c r="A1401" t="n">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="1402">
-      <c r="A1402" t="n">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="1403">
-      <c r="A1403" t="n">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="1404">
-      <c r="A1404" t="n">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="1405">
-      <c r="A1405" t="n">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="1406">
-      <c r="A1406" t="n">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="1407">
-      <c r="A1407" t="n">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="1408">
-      <c r="A1408" t="n">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="1409">
-      <c r="A1409" t="n">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="1410">
-      <c r="A1410" t="n">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="1411">
-      <c r="A1411" t="n">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="1412">
-      <c r="A1412" t="n">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="1413">
-      <c r="A1413" t="n">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="1414">
-      <c r="A1414" t="n">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="1415">
-      <c r="A1415" t="n">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="1416">
-      <c r="A1416" t="n">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="1417">
-      <c r="A1417" t="n">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="1418">
-      <c r="A1418" t="n">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="1419">
-      <c r="A1419" t="n">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="1420">
-      <c r="A1420" t="n">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="1421">
-      <c r="A1421" t="n">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="1422">
-      <c r="A1422" t="n">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="1423">
-      <c r="A1423" t="n">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="1424">
-      <c r="A1424" t="n">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="1425">
-      <c r="A1425" t="n">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="1426">
-      <c r="A1426" t="n">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="1427">
-      <c r="A1427" t="n">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="1428">
-      <c r="A1428" t="n">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="1429">
-      <c r="A1429" t="n">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="1430">
-      <c r="A1430" t="n">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="1431">
-      <c r="A1431" t="n">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="1432">
-      <c r="A1432" t="n">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="1433">
-      <c r="A1433" t="n">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="1434">
-      <c r="A1434" t="n">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="1435">
-      <c r="A1435" t="n">
-        <v>4</v>
-      </c>
-    </row>
   </sheetData>
-  <autoFilter ref="A1:M1435"/>
+  <autoFilter ref="A1:M1049"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Filter to valid units only, normalize GSTerr refs, add CHANGES log
</commit_message>
<xml_diff>
--- a/terrestrial/Towards_SDS/Terrestrial_Master_SDS-aligned.xlsx
+++ b/terrestrial/Towards_SDS/Terrestrial_Master_SDS-aligned.xlsx
@@ -10,7 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="tblGeoschemesTerrestrial" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'tblGeoschemesTerrestrial'!$A$1:$M$1049</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'tblGeoschemesTerrestrial'!$A$1:$M$1048</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -428,7 +428,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M1049"/>
+  <dimension ref="A1:M1048"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -27321,7 +27321,7 @@
       </c>
       <c r="K903" t="inlineStr">
         <is>
-          <t>New unit, split from PAL-IS per GSTerr9.</t>
+          <t>New unit, split from PAL-IS per issue #10.</t>
         </is>
       </c>
       <c r="L903" t="inlineStr">
@@ -27361,7 +27361,7 @@
       </c>
       <c r="K904" t="inlineStr">
         <is>
-          <t>Redefined per GSTerr9: previously included Gaza Strip and West Bank (WGSRPD ed. 2 limits); now split into PAL-GZ and PAL-WB.</t>
+          <t>Redefined per issue #10: previously included Gaza Strip and West Bank (WGSRPD ed. 2 limits); now split into PAL-GZ and PAL-WB.</t>
         </is>
       </c>
       <c r="L904" t="inlineStr">
@@ -27431,7 +27431,7 @@
       </c>
       <c r="K906" t="inlineStr">
         <is>
-          <t>New unit, split from PAL-IS per GSTerr9.</t>
+          <t>New unit, split from PAL-IS per issue #10.</t>
         </is>
       </c>
       <c r="L906" t="inlineStr">
@@ -31909,53 +31909,8 @@
         </is>
       </c>
     </row>
-    <row r="1049">
-      <c r="A1049" t="n">
-        <v>4</v>
-      </c>
-      <c r="B1049" t="inlineStr">
-        <is>
-          <t>SUD-OO</t>
-        </is>
-      </c>
-      <c r="C1049" t="inlineStr">
-        <is>
-          <t>Sudan</t>
-        </is>
-      </c>
-      <c r="D1049" t="inlineStr">
-        <is>
-          <t>SUD</t>
-        </is>
-      </c>
-      <c r="E1049" t="inlineStr">
-        <is>
-          <t>SD</t>
-        </is>
-      </c>
-      <c r="F1049" t="inlineStr">
-        <is>
-          <t>SUD_OO</t>
-        </is>
-      </c>
-      <c r="H1049" t="inlineStr">
-        <is>
-          <t>D</t>
-        </is>
-      </c>
-      <c r="I1049" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="L1049" t="inlineStr">
-        <is>
-          <t>#11</t>
-        </is>
-      </c>
-    </row>
   </sheetData>
-  <autoFilter ref="A1:M1049"/>
+  <autoFilter ref="A1:M1048"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Remove Id column from master table
</commit_message>
<xml_diff>
--- a/terrestrial/Towards_SDS/Terrestrial_Master_SDS-aligned.xlsx
+++ b/terrestrial/Towards_SDS/Terrestrial_Master_SDS-aligned.xlsx
@@ -10,7 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="tblGeoschemesTerrestrial" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'tblGeoschemesTerrestrial'!$A$1:$N$1048</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'tblGeoschemesTerrestrial'!$A$1:$M$1048</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -428,7 +428,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N1048"/>
+  <dimension ref="A1:M1048"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -444,7 +444,6 @@
     <col width="7" customWidth="1" min="11" max="11"/>
     <col width="9" customWidth="1" min="12" max="12"/>
     <col width="16" customWidth="1" min="13" max="13"/>
-    <col width="6" customWidth="1" min="14" max="14"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -514,11 +513,6 @@
           <t>Change according to page 9</t>
         </is>
       </c>
-      <c r="N1" s="1" t="inlineStr">
-        <is>
-          <t>Id</t>
-        </is>
-      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -544,9 +538,6 @@
       <c r="K2" t="n">
         <v>1</v>
       </c>
-      <c r="N2" t="n">
-        <v>1</v>
-      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -572,9 +563,6 @@
       <c r="K3" t="n">
         <v>1</v>
       </c>
-      <c r="N3" t="n">
-        <v>2</v>
-      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -600,9 +588,6 @@
       <c r="K4" t="n">
         <v>1</v>
       </c>
-      <c r="N4" t="n">
-        <v>3</v>
-      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -628,9 +613,6 @@
       <c r="K5" t="n">
         <v>1</v>
       </c>
-      <c r="N5" t="n">
-        <v>4</v>
-      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -656,9 +638,6 @@
       <c r="K6" t="n">
         <v>1</v>
       </c>
-      <c r="N6" t="n">
-        <v>5</v>
-      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -684,9 +663,6 @@
       <c r="K7" t="n">
         <v>1</v>
       </c>
-      <c r="N7" t="n">
-        <v>6</v>
-      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -712,9 +688,6 @@
       <c r="K8" t="n">
         <v>1</v>
       </c>
-      <c r="N8" t="n">
-        <v>7</v>
-      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -740,9 +713,6 @@
       <c r="K9" t="n">
         <v>1</v>
       </c>
-      <c r="N9" t="n">
-        <v>8</v>
-      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -767,9 +737,6 @@
       </c>
       <c r="K10" t="n">
         <v>1</v>
-      </c>
-      <c r="N10" t="n">
-        <v>9</v>
       </c>
     </row>
     <row r="11">
@@ -42651,7 +42618,7 @@
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:N1048"/>
+  <autoFilter ref="A1:M1048"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>